<commit_message>
Standardize priority options to High, Medium, Low across UI, backend, and Excel
</commit_message>
<xml_diff>
--- a/ServiceRequestReport-639195597679312838 (2).xlsx
+++ b/ServiceRequestReport-639195597679312838 (2).xlsx
@@ -1,25 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ishdupso1\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11880"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet sheetId="2" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="110">
   <si>
     <t>ServiceRequestId</t>
   </si>
@@ -69,25 +64,85 @@
     <t>Part No./Part Description</t>
   </si>
   <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>RESOLUTION</t>
+  </si>
+  <si>
+    <t>SR0306202620776</t>
+  </si>
+  <si>
+    <t>03-06-2026</t>
+  </si>
+  <si>
     <t>UTTAR PRADESH</t>
   </si>
   <si>
     <t>LUCKNOW-MARKETING</t>
   </si>
   <si>
+    <t>Engineer Visit Required</t>
+  </si>
+  <si>
+    <t>Desktop Engineer Required</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>PC BOOTING ISSUEOS CORRUPTED</t>
+  </si>
+  <si>
+    <t>MIRZAPUER TERMINAL - ARUN  KUMAR BHARTI</t>
+  </si>
+  <si>
+    <t>ARUN KUMAR BHARTI  IOCL MARKETING  MIRZAPUR TERMINAL  VILL HINAUTI SADAR TEHSIL NR SANTUSTI AYURVEDIC MED COLLEGE  MIRZAPUR  CHUNAR  MIRZAPUR  (UTTAR PRADESH )-231304</t>
+  </si>
+  <si>
+    <t>Haritosh Mishra</t>
+  </si>
+  <si>
+    <t>OS NEED TO BE REINSTALL.</t>
+  </si>
+  <si>
+    <t>UXVTUSI512M5096222</t>
+  </si>
+  <si>
+    <t>ACER</t>
+  </si>
+  <si>
+    <t>ACER VERITON M200 - P565</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>SR1006202621062</t>
+  </si>
+  <si>
+    <t>10-06-2026</t>
+  </si>
+  <si>
     <t>Desktop</t>
   </si>
   <si>
     <t>Keyboard</t>
   </si>
   <si>
-    <t>Medium</t>
-  </si>
-  <si>
     <t>USB KEYBOARD &amp; USB MOUSE NOT WORKING</t>
   </si>
   <si>
-    <t>Haritosh Mishra</t>
+    <t>VARANASI DO - GUNJAN KUMAR</t>
+  </si>
+  <si>
+    <t>MR RAM KUMAR SHUKLA INDIAN OIL CORPORATION LTD  (MD)  INDANE BOTTLING PLANT  NH-31  BABATPUR ROAD  HARAHUA  VARANASI - 221105. MOB:-  7754998889</t>
+  </si>
+  <si>
+    <t>USB KEYBOARD &amp; MOUSE ISSUE</t>
+  </si>
+  <si>
+    <t>INA916R013</t>
   </si>
   <si>
     <t>HP</t>
@@ -96,210 +151,156 @@
     <t>HP PRODESK 600</t>
   </si>
   <si>
+    <t>USB KEYBOARD  and  USB MOUSE</t>
+  </si>
+  <si>
+    <t>SR1706202621349</t>
+  </si>
+  <si>
+    <t>17-06-2026</t>
+  </si>
+  <si>
+    <t>VARANASI AO - MUKHLISA MARIYAM</t>
+  </si>
+  <si>
+    <t>USB KEYBOARD &amp; USB MOUSE ISSUE</t>
+  </si>
+  <si>
+    <t>ACL05635</t>
+  </si>
+  <si>
+    <t>ACXXEL</t>
+  </si>
+  <si>
+    <t>ACXXEL  I7</t>
+  </si>
+  <si>
+    <t>SR1706202621351</t>
+  </si>
+  <si>
+    <t>KANPUR DO - GAURAV VERMA</t>
+  </si>
+  <si>
+    <t>MR PRABHAKAR INDIAN OIL CORPORATION LTD. (MD)  BULK TERMINAL  KALPI ROAD  PANKI  KANPUR - 208020 (U.P.). MOB:  9935984111</t>
+  </si>
+  <si>
+    <t>UXVTUSI512M5095935</t>
+  </si>
+  <si>
+    <t>SR1706202621352</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>KANPUR DO - ADARSH SACHAN</t>
+  </si>
+  <si>
+    <t>UXVTUSI512M5095908</t>
+  </si>
+  <si>
+    <t>SR2606202621857</t>
+  </si>
+  <si>
+    <t>26-06-2026</t>
+  </si>
+  <si>
+    <t>VARANASI AO - NITESH KUMAR</t>
+  </si>
+  <si>
+    <t>UXVTUSI512M5096258</t>
+  </si>
+  <si>
+    <t>SR2606202621858</t>
+  </si>
+  <si>
     <t>HDD</t>
   </si>
   <si>
     <t>OS NOT GETTING INSTALLED</t>
   </si>
   <si>
+    <t>STATE OFFICE - AFTAB AHMED</t>
+  </si>
+  <si>
     <t>HARITOSH MISHRA  INDIAN OIL CORPORATION LIMITED   (MD) UP STATE OFFICE 1  INDIAN OIL BHAVAN  TC-39/V  VIBHUTI KHAND  GOMTI NAGAR  LUCKNOW UTTAR PRADESH -226010 MOB: 9956172789</t>
   </si>
   <si>
     <t>1 TB SATA HDD ISSUE</t>
   </si>
   <si>
+    <t>INA916R03Y</t>
+  </si>
+  <si>
     <t>1 TB SATA HDD</t>
   </si>
   <si>
+    <t>SR2606202621860</t>
+  </si>
+  <si>
     <t>High</t>
   </si>
   <si>
     <t>WIRELESS KBD &amp; MOUSE NOT WORKING</t>
   </si>
   <si>
+    <t>STATE OFFICE - RAJESH  GUPTA</t>
+  </si>
+  <si>
+    <t>4J5LBV3</t>
+  </si>
+  <si>
     <t>DELL</t>
   </si>
   <si>
     <t>DELL OPTIPLEX 5400 AIO</t>
   </si>
   <si>
-    <t>ACER</t>
-  </si>
-  <si>
-    <t>ACER VERITON M200 - P565</t>
+    <t>WIRELESS KEYBOARD  and  MOUSE</t>
+  </si>
+  <si>
+    <t>SR0607202622183</t>
+  </si>
+  <si>
+    <t>06-07-2026</t>
+  </si>
+  <si>
+    <t>VARANASI BP - KISHAN KUMAR</t>
+  </si>
+  <si>
+    <t>UXVTUSI512M5095745</t>
+  </si>
+  <si>
+    <t>SR0607202622184</t>
+  </si>
+  <si>
+    <t>VARANASI AO - RAJAT KUMAR</t>
+  </si>
+  <si>
+    <t>ACL05631</t>
+  </si>
+  <si>
+    <t>SR0607202622220</t>
+  </si>
+  <si>
+    <t>MUGALSARAI TERMINAL - AMAR SINGH</t>
+  </si>
+  <si>
+    <t>1 TB  SATA HDD DETECTION ISSUE</t>
+  </si>
+  <si>
+    <t>INA916R045</t>
+  </si>
+  <si>
+    <t>SR0707202622259</t>
+  </si>
+  <si>
+    <t>07-07-2026</t>
   </si>
   <si>
     <t>Motherboard</t>
   </si>
   <si>
-    <t>Engineer Visit Required</t>
-  </si>
-  <si>
-    <t>Desktop Engineer Required</t>
-  </si>
-  <si>
-    <t>MR RAM KUMAR SHUKLA INDIAN OIL CORPORATION LTD  (MD)  INDANE BOTTLING PLANT  NH-31  BABATPUR ROAD  HARAHUA  VARANASI - 221105. MOB:-  7754998889</t>
-  </si>
-  <si>
-    <t>03-06-2026</t>
-  </si>
-  <si>
-    <t>USB KEYBOARD &amp; MOUSE ISSUE</t>
-  </si>
-  <si>
-    <t>SR0306202620776</t>
-  </si>
-  <si>
-    <t>PC BOOTING ISSUEOS CORRUPTED</t>
-  </si>
-  <si>
-    <t>MIRZAPUER TERMINAL - ARUN  KUMAR BHARTI</t>
-  </si>
-  <si>
-    <t>ARUN KUMAR BHARTI  IOCL MARKETING  MIRZAPUR TERMINAL  VILL HINAUTI SADAR TEHSIL NR SANTUSTI AYURVEDIC MED COLLEGE  MIRZAPUR  CHUNAR  MIRZAPUR  (UTTAR PRADESH )-231304</t>
-  </si>
-  <si>
-    <t>OS NEED TO BE REINSTALL.</t>
-  </si>
-  <si>
-    <t>UXVTUSI512M5096222</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>SR1006202621062</t>
-  </si>
-  <si>
-    <t>10-06-2026</t>
-  </si>
-  <si>
-    <t>VARANASI DO - GUNJAN KUMAR</t>
-  </si>
-  <si>
-    <t>INA916R013</t>
-  </si>
-  <si>
-    <t>USB KEYBOARD  and  USB MOUSE</t>
-  </si>
-  <si>
-    <t>SR1706202621349</t>
-  </si>
-  <si>
-    <t>17-06-2026</t>
-  </si>
-  <si>
-    <t>VARANASI AO - MUKHLISA MARIYAM</t>
-  </si>
-  <si>
-    <t>USB KEYBOARD &amp; USB MOUSE ISSUE</t>
-  </si>
-  <si>
-    <t>ACL05635</t>
-  </si>
-  <si>
-    <t>ACXXEL</t>
-  </si>
-  <si>
-    <t>ACXXEL  I7</t>
-  </si>
-  <si>
-    <t>SR1706202621351</t>
-  </si>
-  <si>
-    <t>KANPUR DO - GAURAV VERMA</t>
-  </si>
-  <si>
-    <t>MR PRABHAKAR INDIAN OIL CORPORATION LTD. (MD)  BULK TERMINAL  KALPI ROAD  PANKI  KANPUR - 208020 (U.P.). MOB:  9935984111</t>
-  </si>
-  <si>
-    <t>UXVTUSI512M5095935</t>
-  </si>
-  <si>
-    <t>SR1706202621352</t>
-  </si>
-  <si>
-    <t>Very Low</t>
-  </si>
-  <si>
-    <t>KANPUR DO - ADARSH SACHAN</t>
-  </si>
-  <si>
-    <t>UXVTUSI512M5095908</t>
-  </si>
-  <si>
-    <t>SR2606202621857</t>
-  </si>
-  <si>
-    <t>26-06-2026</t>
-  </si>
-  <si>
-    <t>VARANASI AO - NITESH KUMAR</t>
-  </si>
-  <si>
-    <t>UXVTUSI512M5096258</t>
-  </si>
-  <si>
-    <t>SR2606202621858</t>
-  </si>
-  <si>
-    <t>STATE OFFICE - AFTAB AHMED</t>
-  </si>
-  <si>
-    <t>INA916R03Y</t>
-  </si>
-  <si>
-    <t>06-07-2026</t>
-  </si>
-  <si>
-    <t>SR2606202621860</t>
-  </si>
-  <si>
-    <t>STATE OFFICE - RAJESH  GUPTA</t>
-  </si>
-  <si>
-    <t>4J5LBV3</t>
-  </si>
-  <si>
-    <t>WIRELESS KEYBOARD  and  MOUSE</t>
-  </si>
-  <si>
-    <t>SR0607202622183</t>
-  </si>
-  <si>
-    <t>VARANASI BP - KISHAN KUMAR</t>
-  </si>
-  <si>
-    <t>UXVTUSI512M5095745</t>
-  </si>
-  <si>
-    <t>SR0607202622184</t>
-  </si>
-  <si>
-    <t>VARANASI AO - RAJAT KUMAR</t>
-  </si>
-  <si>
-    <t>ACL05631</t>
-  </si>
-  <si>
-    <t>SR0607202622220</t>
-  </si>
-  <si>
-    <t>MUGALSARAI TERMINAL - AMAR SINGH</t>
-  </si>
-  <si>
-    <t>1 TB  SATA HDD DETECTION ISSUE</t>
-  </si>
-  <si>
-    <t>INA916R045</t>
-  </si>
-  <si>
-    <t>SR0707202622259</t>
-  </si>
-  <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
     <t>PC NO DISPLAY</t>
   </si>
   <si>
@@ -313,6 +314,36 @@
   </si>
   <si>
     <t>ACER PRO565AM4-M9 /Supports AMD AM4 socket for AMD Ryzen™ processors</t>
+  </si>
+  <si>
+    <t>SR-TEST-VERIFY</t>
+  </si>
+  <si>
+    <t>28/09/2026</t>
+  </si>
+  <si>
+    <t>UPSO-I, Lucknow</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test complaint</t>
+  </si>
+  <si>
+    <t>SR-420929-4948</t>
+  </si>
+  <si>
+    <t>UPSO-1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>54606318</t>
+  </si>
+  <si>
+    <t>New</t>
   </si>
 </sst>
 </file>
@@ -321,10 +352,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -345,10 +377,10 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -367,8 +399,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:P13" totalsRowShown="0">
-  <autoFilter ref="A1:P13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Table1" displayName="Table1" ref="A1:P13" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P13">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
     <tableColumn id="1" name="ServiceRequestId"/>
     <tableColumn id="2" name="Logged Date"/>
@@ -674,10 +723,10 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" customWidth="1"/>
@@ -694,10 +743,10 @@
     <col min="13" max="13" width="26.85546875" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
     <col min="15" max="15" width="25.7109375" customWidth="1"/>
-    <col min="16" max="16" width="96.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="96.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -745,403 +794,409 @@
       </c>
       <c r="P1" t="s">
         <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="M2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="N2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="J3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L3" t="s">
         <v>41</v>
       </c>
       <c r="M3" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="O3" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="P3" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K4" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="N4" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="O4" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="P4" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" t="s">
         <v>55</v>
       </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J5" t="s">
-        <v>63</v>
-      </c>
       <c r="K5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="N5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P5" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J6" t="s">
         <v>55</v>
       </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" t="s">
-        <v>67</v>
-      </c>
-      <c r="J6" t="s">
-        <v>63</v>
-      </c>
       <c r="K6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="M6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="N6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P6" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="J7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K7" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L7" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="M7" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="N7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P7" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" t="s">
+        <v>67</v>
+      </c>
+      <c r="I8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K8" t="s">
+        <v>28</v>
+      </c>
+      <c r="L8" t="s">
         <v>70</v>
       </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" t="s">
-        <v>74</v>
-      </c>
-      <c r="J8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" t="s">
-        <v>28</v>
-      </c>
       <c r="M8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N8" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="O8" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="P8" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>74</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" t="s">
+        <v>75</v>
+      </c>
+      <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="B9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="N9" t="s">
         <v>78</v>
       </c>
-      <c r="J9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K9" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" t="s">
-        <v>31</v>
-      </c>
-      <c r="M9" t="s">
+      <c r="O9" t="s">
         <v>79</v>
-      </c>
-      <c r="N9" t="s">
-        <v>32</v>
-      </c>
-      <c r="O9" t="s">
-        <v>33</v>
       </c>
       <c r="P9" t="s">
         <v>80</v>
@@ -1152,199 +1207,263 @@
         <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K10" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L10" t="s">
         <v>41</v>
       </c>
       <c r="M10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="N10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P10" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="I11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L11" t="s">
         <v>41</v>
       </c>
       <c r="M11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N11" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="O11" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="P11" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="H12" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="I12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K12" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="N12" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="O12" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="P12" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>36</v>
+        <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="H13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J13" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="K13" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="L13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="N13" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="P13" t="s">
-        <v>97</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" t="s">
+        <v>103</v>
+      </c>
+      <c r="F15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" t="s">
+        <v>107</v>
+      </c>
+      <c r="K15" t="s">
+        <v>107</v>
+      </c>
+      <c r="L15" t="s">
+        <v>103</v>
+      </c>
+      <c r="M15" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>109</v>
+      </c>
+      <c r="R15" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>